<commit_message>
Support income and expense cash flow imports
</commit_message>
<xml_diff>
--- a/public/templates/cash-flow-import-template.xlsx
+++ b/public/templates/cash-flow-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="1" r:id="R5488cd7a57be45cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R14e31d8916b14cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="1" r:id="R2f4cad4abd784c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rbafba1610bd84163"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -373,9 +373,9 @@
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -386,16 +386,16 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Description</x:v>
+        <x:v>Service Description</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Amount (PKR)</x:v>
+        <x:v>Income Intake Amount</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Payment Method</x:v>
+        <x:v>Expense Amount</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Notes</x:v>
+        <x:v>Closing</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -403,19 +403,20 @@
         <x:v>46174.291666666664</x:v>
       </x:c>
       <x:c r="B2" s="14" t="str">
-        <x:v>Rent</x:v>
+        <x:v>Services</x:v>
       </x:c>
       <x:c r="C2" s="22" t="str">
-        <x:v>Monthly salon rent</x:v>
+        <x:v>Hair service income</x:v>
       </x:c>
       <x:c r="D2" s="15" t="n">
-        <x:v>85000</x:v>
-      </x:c>
-      <x:c r="E2" s="14" t="str">
-        <x:v>Bank Transfer</x:v>
-      </x:c>
-      <x:c r="F2" s="22" t="str">
-        <x:v>June rent</x:v>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="E2" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="15" t="n">
+        <x:f>D2-E2</x:f>
+        <x:v>12000</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -426,16 +427,17 @@
         <x:v>Products &amp; Supplies</x:v>
       </x:c>
       <x:c r="C3" s="23" t="str">
-        <x:v>Shampoo and conditioner restock</x:v>
+        <x:v>Shampoo restock</x:v>
       </x:c>
       <x:c r="D3" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="n">
         <x:v>24500</x:v>
       </x:c>
-      <x:c r="E3" s="17" t="str">
-        <x:v>Cash</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>Supplier invoice 1042</x:v>
+      <x:c r="F3" s="18" t="n">
+        <x:f>D3-E3</x:f>
+        <x:v>-24500</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -449,1588 +451,2176 @@
         <x:v>Electricity bill</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="18" t="n">
         <x:v>18000</x:v>
       </x:c>
-      <x:c r="E4" s="17" t="str">
-        <x:v>JazzCash</x:v>
-      </x:c>
-      <x:c r="F4" s="23" t="str"/>
+      <x:c r="F4" s="18" t="n">
+        <x:f>D4-E4</x:f>
+        <x:v>-18000</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16"/>
       <x:c r="B5" s="17"/>
       <x:c r="C5" s="23"/>
       <x:c r="D5" s="18"/>
-      <x:c r="E5" s="17"/>
-      <x:c r="F5" s="23"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18" t="n">
+        <x:f>D5-E5</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16"/>
       <x:c r="B6" s="17"/>
       <x:c r="C6" s="23"/>
       <x:c r="D6" s="18"/>
-      <x:c r="E6" s="17"/>
-      <x:c r="F6" s="23"/>
+      <x:c r="E6" s="18"/>
+      <x:c r="F6" s="18" t="n">
+        <x:f>D6-E6</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16"/>
       <x:c r="B7" s="17"/>
       <x:c r="C7" s="23"/>
       <x:c r="D7" s="18"/>
-      <x:c r="E7" s="17"/>
-      <x:c r="F7" s="23"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18" t="n">
+        <x:f>D7-E7</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16"/>
       <x:c r="B8" s="17"/>
       <x:c r="C8" s="23"/>
       <x:c r="D8" s="18"/>
-      <x:c r="E8" s="17"/>
-      <x:c r="F8" s="23"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18" t="n">
+        <x:f>D8-E8</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16"/>
       <x:c r="B9" s="17"/>
       <x:c r="C9" s="23"/>
       <x:c r="D9" s="18"/>
-      <x:c r="E9" s="17"/>
-      <x:c r="F9" s="23"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18" t="n">
+        <x:f>D9-E9</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16"/>
       <x:c r="B10" s="17"/>
       <x:c r="C10" s="23"/>
       <x:c r="D10" s="18"/>
-      <x:c r="E10" s="17"/>
-      <x:c r="F10" s="23"/>
+      <x:c r="E10" s="18"/>
+      <x:c r="F10" s="18" t="n">
+        <x:f>D10-E10</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16"/>
       <x:c r="B11" s="17"/>
       <x:c r="C11" s="23"/>
       <x:c r="D11" s="18"/>
-      <x:c r="E11" s="17"/>
-      <x:c r="F11" s="23"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18" t="n">
+        <x:f>D11-E11</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16"/>
       <x:c r="B12" s="17"/>
       <x:c r="C12" s="23"/>
       <x:c r="D12" s="18"/>
-      <x:c r="E12" s="17"/>
-      <x:c r="F12" s="23"/>
+      <x:c r="E12" s="18"/>
+      <x:c r="F12" s="18" t="n">
+        <x:f>D12-E12</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16"/>
       <x:c r="B13" s="17"/>
       <x:c r="C13" s="23"/>
       <x:c r="D13" s="18"/>
-      <x:c r="E13" s="17"/>
-      <x:c r="F13" s="23"/>
+      <x:c r="E13" s="18"/>
+      <x:c r="F13" s="18" t="n">
+        <x:f>D13-E13</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="16"/>
       <x:c r="B14" s="17"/>
       <x:c r="C14" s="23"/>
       <x:c r="D14" s="18"/>
-      <x:c r="E14" s="17"/>
-      <x:c r="F14" s="23"/>
+      <x:c r="E14" s="18"/>
+      <x:c r="F14" s="18" t="n">
+        <x:f>D14-E14</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="16"/>
       <x:c r="B15" s="17"/>
       <x:c r="C15" s="23"/>
       <x:c r="D15" s="18"/>
-      <x:c r="E15" s="17"/>
-      <x:c r="F15" s="23"/>
+      <x:c r="E15" s="18"/>
+      <x:c r="F15" s="18" t="n">
+        <x:f>D15-E15</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="16"/>
       <x:c r="B16" s="17"/>
       <x:c r="C16" s="23"/>
       <x:c r="D16" s="18"/>
-      <x:c r="E16" s="17"/>
-      <x:c r="F16" s="23"/>
+      <x:c r="E16" s="18"/>
+      <x:c r="F16" s="18" t="n">
+        <x:f>D16-E16</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="16"/>
       <x:c r="B17" s="17"/>
       <x:c r="C17" s="23"/>
       <x:c r="D17" s="18"/>
-      <x:c r="E17" s="17"/>
-      <x:c r="F17" s="23"/>
+      <x:c r="E17" s="18"/>
+      <x:c r="F17" s="18" t="n">
+        <x:f>D17-E17</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="16"/>
       <x:c r="B18" s="17"/>
       <x:c r="C18" s="23"/>
       <x:c r="D18" s="18"/>
-      <x:c r="E18" s="17"/>
-      <x:c r="F18" s="23"/>
+      <x:c r="E18" s="18"/>
+      <x:c r="F18" s="18" t="n">
+        <x:f>D18-E18</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="16"/>
       <x:c r="B19" s="17"/>
       <x:c r="C19" s="23"/>
       <x:c r="D19" s="18"/>
-      <x:c r="E19" s="17"/>
-      <x:c r="F19" s="23"/>
+      <x:c r="E19" s="18"/>
+      <x:c r="F19" s="18" t="n">
+        <x:f>D19-E19</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="16"/>
       <x:c r="B20" s="17"/>
       <x:c r="C20" s="23"/>
       <x:c r="D20" s="18"/>
-      <x:c r="E20" s="17"/>
-      <x:c r="F20" s="23"/>
+      <x:c r="E20" s="18"/>
+      <x:c r="F20" s="18" t="n">
+        <x:f>D20-E20</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="16"/>
       <x:c r="B21" s="17"/>
       <x:c r="C21" s="23"/>
       <x:c r="D21" s="18"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="23"/>
+      <x:c r="E21" s="18"/>
+      <x:c r="F21" s="18" t="n">
+        <x:f>D21-E21</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="16"/>
       <x:c r="B22" s="17"/>
       <x:c r="C22" s="23"/>
       <x:c r="D22" s="18"/>
-      <x:c r="E22" s="17"/>
-      <x:c r="F22" s="23"/>
+      <x:c r="E22" s="18"/>
+      <x:c r="F22" s="18" t="n">
+        <x:f>D22-E22</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="16"/>
       <x:c r="B23" s="17"/>
       <x:c r="C23" s="23"/>
       <x:c r="D23" s="18"/>
-      <x:c r="E23" s="17"/>
-      <x:c r="F23" s="23"/>
+      <x:c r="E23" s="18"/>
+      <x:c r="F23" s="18" t="n">
+        <x:f>D23-E23</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="16"/>
       <x:c r="B24" s="17"/>
       <x:c r="C24" s="23"/>
       <x:c r="D24" s="18"/>
-      <x:c r="E24" s="17"/>
-      <x:c r="F24" s="23"/>
+      <x:c r="E24" s="18"/>
+      <x:c r="F24" s="18" t="n">
+        <x:f>D24-E24</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="16"/>
       <x:c r="B25" s="17"/>
       <x:c r="C25" s="23"/>
       <x:c r="D25" s="18"/>
-      <x:c r="E25" s="17"/>
-      <x:c r="F25" s="23"/>
+      <x:c r="E25" s="18"/>
+      <x:c r="F25" s="18" t="n">
+        <x:f>D25-E25</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="16"/>
       <x:c r="B26" s="17"/>
       <x:c r="C26" s="23"/>
       <x:c r="D26" s="18"/>
-      <x:c r="E26" s="17"/>
-      <x:c r="F26" s="23"/>
+      <x:c r="E26" s="18"/>
+      <x:c r="F26" s="18" t="n">
+        <x:f>D26-E26</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="16"/>
       <x:c r="B27" s="17"/>
       <x:c r="C27" s="23"/>
       <x:c r="D27" s="18"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="23"/>
+      <x:c r="E27" s="18"/>
+      <x:c r="F27" s="18" t="n">
+        <x:f>D27-E27</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="16"/>
       <x:c r="B28" s="17"/>
       <x:c r="C28" s="23"/>
       <x:c r="D28" s="18"/>
-      <x:c r="E28" s="17"/>
-      <x:c r="F28" s="23"/>
+      <x:c r="E28" s="18"/>
+      <x:c r="F28" s="18" t="n">
+        <x:f>D28-E28</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="16"/>
       <x:c r="B29" s="17"/>
       <x:c r="C29" s="23"/>
       <x:c r="D29" s="18"/>
-      <x:c r="E29" s="17"/>
-      <x:c r="F29" s="23"/>
+      <x:c r="E29" s="18"/>
+      <x:c r="F29" s="18" t="n">
+        <x:f>D29-E29</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="16"/>
       <x:c r="B30" s="17"/>
       <x:c r="C30" s="23"/>
       <x:c r="D30" s="18"/>
-      <x:c r="E30" s="17"/>
-      <x:c r="F30" s="23"/>
+      <x:c r="E30" s="18"/>
+      <x:c r="F30" s="18" t="n">
+        <x:f>D30-E30</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="16"/>
       <x:c r="B31" s="17"/>
       <x:c r="C31" s="23"/>
       <x:c r="D31" s="18"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="23"/>
+      <x:c r="E31" s="18"/>
+      <x:c r="F31" s="18" t="n">
+        <x:f>D31-E31</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="16"/>
       <x:c r="B32" s="17"/>
       <x:c r="C32" s="23"/>
       <x:c r="D32" s="18"/>
-      <x:c r="E32" s="17"/>
-      <x:c r="F32" s="23"/>
+      <x:c r="E32" s="18"/>
+      <x:c r="F32" s="18" t="n">
+        <x:f>D32-E32</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="16"/>
       <x:c r="B33" s="17"/>
       <x:c r="C33" s="23"/>
       <x:c r="D33" s="18"/>
-      <x:c r="E33" s="17"/>
-      <x:c r="F33" s="23"/>
+      <x:c r="E33" s="18"/>
+      <x:c r="F33" s="18" t="n">
+        <x:f>D33-E33</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="16"/>
       <x:c r="B34" s="17"/>
       <x:c r="C34" s="23"/>
       <x:c r="D34" s="18"/>
-      <x:c r="E34" s="17"/>
-      <x:c r="F34" s="23"/>
+      <x:c r="E34" s="18"/>
+      <x:c r="F34" s="18" t="n">
+        <x:f>D34-E34</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="16"/>
       <x:c r="B35" s="17"/>
       <x:c r="C35" s="23"/>
       <x:c r="D35" s="18"/>
-      <x:c r="E35" s="17"/>
-      <x:c r="F35" s="23"/>
+      <x:c r="E35" s="18"/>
+      <x:c r="F35" s="18" t="n">
+        <x:f>D35-E35</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="16"/>
       <x:c r="B36" s="17"/>
       <x:c r="C36" s="23"/>
       <x:c r="D36" s="18"/>
-      <x:c r="E36" s="17"/>
-      <x:c r="F36" s="23"/>
+      <x:c r="E36" s="18"/>
+      <x:c r="F36" s="18" t="n">
+        <x:f>D36-E36</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="16"/>
       <x:c r="B37" s="17"/>
       <x:c r="C37" s="23"/>
       <x:c r="D37" s="18"/>
-      <x:c r="E37" s="17"/>
-      <x:c r="F37" s="23"/>
+      <x:c r="E37" s="18"/>
+      <x:c r="F37" s="18" t="n">
+        <x:f>D37-E37</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="16"/>
       <x:c r="B38" s="17"/>
       <x:c r="C38" s="23"/>
       <x:c r="D38" s="18"/>
-      <x:c r="E38" s="17"/>
-      <x:c r="F38" s="23"/>
+      <x:c r="E38" s="18"/>
+      <x:c r="F38" s="18" t="n">
+        <x:f>D38-E38</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="16"/>
       <x:c r="B39" s="17"/>
       <x:c r="C39" s="23"/>
       <x:c r="D39" s="18"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="23"/>
+      <x:c r="E39" s="18"/>
+      <x:c r="F39" s="18" t="n">
+        <x:f>D39-E39</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="16"/>
       <x:c r="B40" s="17"/>
       <x:c r="C40" s="23"/>
       <x:c r="D40" s="18"/>
-      <x:c r="E40" s="17"/>
-      <x:c r="F40" s="23"/>
+      <x:c r="E40" s="18"/>
+      <x:c r="F40" s="18" t="n">
+        <x:f>D40-E40</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="16"/>
       <x:c r="B41" s="17"/>
       <x:c r="C41" s="23"/>
       <x:c r="D41" s="18"/>
-      <x:c r="E41" s="17"/>
-      <x:c r="F41" s="23"/>
+      <x:c r="E41" s="18"/>
+      <x:c r="F41" s="18" t="n">
+        <x:f>D41-E41</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="16"/>
       <x:c r="B42" s="17"/>
       <x:c r="C42" s="23"/>
       <x:c r="D42" s="18"/>
-      <x:c r="E42" s="17"/>
-      <x:c r="F42" s="23"/>
+      <x:c r="E42" s="18"/>
+      <x:c r="F42" s="18" t="n">
+        <x:f>D42-E42</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="16"/>
       <x:c r="B43" s="17"/>
       <x:c r="C43" s="23"/>
       <x:c r="D43" s="18"/>
-      <x:c r="E43" s="17"/>
-      <x:c r="F43" s="23"/>
+      <x:c r="E43" s="18"/>
+      <x:c r="F43" s="18" t="n">
+        <x:f>D43-E43</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="16"/>
       <x:c r="B44" s="17"/>
       <x:c r="C44" s="23"/>
       <x:c r="D44" s="18"/>
-      <x:c r="E44" s="17"/>
-      <x:c r="F44" s="23"/>
+      <x:c r="E44" s="18"/>
+      <x:c r="F44" s="18" t="n">
+        <x:f>D44-E44</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="16"/>
       <x:c r="B45" s="17"/>
       <x:c r="C45" s="23"/>
       <x:c r="D45" s="18"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="23"/>
+      <x:c r="E45" s="18"/>
+      <x:c r="F45" s="18" t="n">
+        <x:f>D45-E45</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="16"/>
       <x:c r="B46" s="17"/>
       <x:c r="C46" s="23"/>
       <x:c r="D46" s="18"/>
-      <x:c r="E46" s="17"/>
-      <x:c r="F46" s="23"/>
+      <x:c r="E46" s="18"/>
+      <x:c r="F46" s="18" t="n">
+        <x:f>D46-E46</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="16"/>
       <x:c r="B47" s="17"/>
       <x:c r="C47" s="23"/>
       <x:c r="D47" s="18"/>
-      <x:c r="E47" s="17"/>
-      <x:c r="F47" s="23"/>
+      <x:c r="E47" s="18"/>
+      <x:c r="F47" s="18" t="n">
+        <x:f>D47-E47</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="16"/>
       <x:c r="B48" s="17"/>
       <x:c r="C48" s="23"/>
       <x:c r="D48" s="18"/>
-      <x:c r="E48" s="17"/>
-      <x:c r="F48" s="23"/>
+      <x:c r="E48" s="18"/>
+      <x:c r="F48" s="18" t="n">
+        <x:f>D48-E48</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="16"/>
       <x:c r="B49" s="17"/>
       <x:c r="C49" s="23"/>
       <x:c r="D49" s="18"/>
-      <x:c r="E49" s="17"/>
-      <x:c r="F49" s="23"/>
+      <x:c r="E49" s="18"/>
+      <x:c r="F49" s="18" t="n">
+        <x:f>D49-E49</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="16"/>
       <x:c r="B50" s="17"/>
       <x:c r="C50" s="23"/>
       <x:c r="D50" s="18"/>
-      <x:c r="E50" s="17"/>
-      <x:c r="F50" s="23"/>
+      <x:c r="E50" s="18"/>
+      <x:c r="F50" s="18" t="n">
+        <x:f>D50-E50</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="16"/>
       <x:c r="B51" s="17"/>
       <x:c r="C51" s="23"/>
       <x:c r="D51" s="18"/>
-      <x:c r="E51" s="17"/>
-      <x:c r="F51" s="23"/>
+      <x:c r="E51" s="18"/>
+      <x:c r="F51" s="18" t="n">
+        <x:f>D51-E51</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="16"/>
       <x:c r="B52" s="17"/>
       <x:c r="C52" s="23"/>
       <x:c r="D52" s="18"/>
-      <x:c r="E52" s="17"/>
-      <x:c r="F52" s="23"/>
+      <x:c r="E52" s="18"/>
+      <x:c r="F52" s="18" t="n">
+        <x:f>D52-E52</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="16"/>
       <x:c r="B53" s="17"/>
       <x:c r="C53" s="23"/>
       <x:c r="D53" s="18"/>
-      <x:c r="E53" s="17"/>
-      <x:c r="F53" s="23"/>
+      <x:c r="E53" s="18"/>
+      <x:c r="F53" s="18" t="n">
+        <x:f>D53-E53</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="16"/>
       <x:c r="B54" s="17"/>
       <x:c r="C54" s="23"/>
       <x:c r="D54" s="18"/>
-      <x:c r="E54" s="17"/>
-      <x:c r="F54" s="23"/>
+      <x:c r="E54" s="18"/>
+      <x:c r="F54" s="18" t="n">
+        <x:f>D54-E54</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="16"/>
       <x:c r="B55" s="17"/>
       <x:c r="C55" s="23"/>
       <x:c r="D55" s="18"/>
-      <x:c r="E55" s="17"/>
-      <x:c r="F55" s="23"/>
+      <x:c r="E55" s="18"/>
+      <x:c r="F55" s="18" t="n">
+        <x:f>D55-E55</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="16"/>
       <x:c r="B56" s="17"/>
       <x:c r="C56" s="23"/>
       <x:c r="D56" s="18"/>
-      <x:c r="E56" s="17"/>
-      <x:c r="F56" s="23"/>
+      <x:c r="E56" s="18"/>
+      <x:c r="F56" s="18" t="n">
+        <x:f>D56-E56</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="16"/>
       <x:c r="B57" s="17"/>
       <x:c r="C57" s="23"/>
       <x:c r="D57" s="18"/>
-      <x:c r="E57" s="17"/>
-      <x:c r="F57" s="23"/>
+      <x:c r="E57" s="18"/>
+      <x:c r="F57" s="18" t="n">
+        <x:f>D57-E57</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="16"/>
       <x:c r="B58" s="17"/>
       <x:c r="C58" s="23"/>
       <x:c r="D58" s="18"/>
-      <x:c r="E58" s="17"/>
-      <x:c r="F58" s="23"/>
+      <x:c r="E58" s="18"/>
+      <x:c r="F58" s="18" t="n">
+        <x:f>D58-E58</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="16"/>
       <x:c r="B59" s="17"/>
       <x:c r="C59" s="23"/>
       <x:c r="D59" s="18"/>
-      <x:c r="E59" s="17"/>
-      <x:c r="F59" s="23"/>
+      <x:c r="E59" s="18"/>
+      <x:c r="F59" s="18" t="n">
+        <x:f>D59-E59</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="16"/>
       <x:c r="B60" s="17"/>
       <x:c r="C60" s="23"/>
       <x:c r="D60" s="18"/>
-      <x:c r="E60" s="17"/>
-      <x:c r="F60" s="23"/>
+      <x:c r="E60" s="18"/>
+      <x:c r="F60" s="18" t="n">
+        <x:f>D60-E60</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="16"/>
       <x:c r="B61" s="17"/>
       <x:c r="C61" s="23"/>
       <x:c r="D61" s="18"/>
-      <x:c r="E61" s="17"/>
-      <x:c r="F61" s="23"/>
+      <x:c r="E61" s="18"/>
+      <x:c r="F61" s="18" t="n">
+        <x:f>D61-E61</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="16"/>
       <x:c r="B62" s="17"/>
       <x:c r="C62" s="23"/>
       <x:c r="D62" s="18"/>
-      <x:c r="E62" s="17"/>
-      <x:c r="F62" s="23"/>
+      <x:c r="E62" s="18"/>
+      <x:c r="F62" s="18" t="n">
+        <x:f>D62-E62</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="16"/>
       <x:c r="B63" s="17"/>
       <x:c r="C63" s="23"/>
       <x:c r="D63" s="18"/>
-      <x:c r="E63" s="17"/>
-      <x:c r="F63" s="23"/>
+      <x:c r="E63" s="18"/>
+      <x:c r="F63" s="18" t="n">
+        <x:f>D63-E63</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="16"/>
       <x:c r="B64" s="17"/>
       <x:c r="C64" s="23"/>
       <x:c r="D64" s="18"/>
-      <x:c r="E64" s="17"/>
-      <x:c r="F64" s="23"/>
+      <x:c r="E64" s="18"/>
+      <x:c r="F64" s="18" t="n">
+        <x:f>D64-E64</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="16"/>
       <x:c r="B65" s="17"/>
       <x:c r="C65" s="23"/>
       <x:c r="D65" s="18"/>
-      <x:c r="E65" s="17"/>
-      <x:c r="F65" s="23"/>
+      <x:c r="E65" s="18"/>
+      <x:c r="F65" s="18" t="n">
+        <x:f>D65-E65</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="16"/>
       <x:c r="B66" s="17"/>
       <x:c r="C66" s="23"/>
       <x:c r="D66" s="18"/>
-      <x:c r="E66" s="17"/>
-      <x:c r="F66" s="23"/>
+      <x:c r="E66" s="18"/>
+      <x:c r="F66" s="18" t="n">
+        <x:f>D66-E66</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="16"/>
       <x:c r="B67" s="17"/>
       <x:c r="C67" s="23"/>
       <x:c r="D67" s="18"/>
-      <x:c r="E67" s="17"/>
-      <x:c r="F67" s="23"/>
+      <x:c r="E67" s="18"/>
+      <x:c r="F67" s="18" t="n">
+        <x:f>D67-E67</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="16"/>
       <x:c r="B68" s="17"/>
       <x:c r="C68" s="23"/>
       <x:c r="D68" s="18"/>
-      <x:c r="E68" s="17"/>
-      <x:c r="F68" s="23"/>
+      <x:c r="E68" s="18"/>
+      <x:c r="F68" s="18" t="n">
+        <x:f>D68-E68</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="16"/>
       <x:c r="B69" s="17"/>
       <x:c r="C69" s="23"/>
       <x:c r="D69" s="18"/>
-      <x:c r="E69" s="17"/>
-      <x:c r="F69" s="23"/>
+      <x:c r="E69" s="18"/>
+      <x:c r="F69" s="18" t="n">
+        <x:f>D69-E69</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="16"/>
       <x:c r="B70" s="17"/>
       <x:c r="C70" s="23"/>
       <x:c r="D70" s="18"/>
-      <x:c r="E70" s="17"/>
-      <x:c r="F70" s="23"/>
+      <x:c r="E70" s="18"/>
+      <x:c r="F70" s="18" t="n">
+        <x:f>D70-E70</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="16"/>
       <x:c r="B71" s="17"/>
       <x:c r="C71" s="23"/>
       <x:c r="D71" s="18"/>
-      <x:c r="E71" s="17"/>
-      <x:c r="F71" s="23"/>
+      <x:c r="E71" s="18"/>
+      <x:c r="F71" s="18" t="n">
+        <x:f>D71-E71</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="16"/>
       <x:c r="B72" s="17"/>
       <x:c r="C72" s="23"/>
       <x:c r="D72" s="18"/>
-      <x:c r="E72" s="17"/>
-      <x:c r="F72" s="23"/>
+      <x:c r="E72" s="18"/>
+      <x:c r="F72" s="18" t="n">
+        <x:f>D72-E72</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="16"/>
       <x:c r="B73" s="17"/>
       <x:c r="C73" s="23"/>
       <x:c r="D73" s="18"/>
-      <x:c r="E73" s="17"/>
-      <x:c r="F73" s="23"/>
+      <x:c r="E73" s="18"/>
+      <x:c r="F73" s="18" t="n">
+        <x:f>D73-E73</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="16"/>
       <x:c r="B74" s="17"/>
       <x:c r="C74" s="23"/>
       <x:c r="D74" s="18"/>
-      <x:c r="E74" s="17"/>
-      <x:c r="F74" s="23"/>
+      <x:c r="E74" s="18"/>
+      <x:c r="F74" s="18" t="n">
+        <x:f>D74-E74</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="16"/>
       <x:c r="B75" s="17"/>
       <x:c r="C75" s="23"/>
       <x:c r="D75" s="18"/>
-      <x:c r="E75" s="17"/>
-      <x:c r="F75" s="23"/>
+      <x:c r="E75" s="18"/>
+      <x:c r="F75" s="18" t="n">
+        <x:f>D75-E75</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="16"/>
       <x:c r="B76" s="17"/>
       <x:c r="C76" s="23"/>
       <x:c r="D76" s="18"/>
-      <x:c r="E76" s="17"/>
-      <x:c r="F76" s="23"/>
+      <x:c r="E76" s="18"/>
+      <x:c r="F76" s="18" t="n">
+        <x:f>D76-E76</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="16"/>
       <x:c r="B77" s="17"/>
       <x:c r="C77" s="23"/>
       <x:c r="D77" s="18"/>
-      <x:c r="E77" s="17"/>
-      <x:c r="F77" s="23"/>
+      <x:c r="E77" s="18"/>
+      <x:c r="F77" s="18" t="n">
+        <x:f>D77-E77</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="16"/>
       <x:c r="B78" s="17"/>
       <x:c r="C78" s="23"/>
       <x:c r="D78" s="18"/>
-      <x:c r="E78" s="17"/>
-      <x:c r="F78" s="23"/>
+      <x:c r="E78" s="18"/>
+      <x:c r="F78" s="18" t="n">
+        <x:f>D78-E78</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="16"/>
       <x:c r="B79" s="17"/>
       <x:c r="C79" s="23"/>
       <x:c r="D79" s="18"/>
-      <x:c r="E79" s="17"/>
-      <x:c r="F79" s="23"/>
+      <x:c r="E79" s="18"/>
+      <x:c r="F79" s="18" t="n">
+        <x:f>D79-E79</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="16"/>
       <x:c r="B80" s="17"/>
       <x:c r="C80" s="23"/>
       <x:c r="D80" s="18"/>
-      <x:c r="E80" s="17"/>
-      <x:c r="F80" s="23"/>
+      <x:c r="E80" s="18"/>
+      <x:c r="F80" s="18" t="n">
+        <x:f>D80-E80</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="16"/>
       <x:c r="B81" s="17"/>
       <x:c r="C81" s="23"/>
       <x:c r="D81" s="18"/>
-      <x:c r="E81" s="17"/>
-      <x:c r="F81" s="23"/>
+      <x:c r="E81" s="18"/>
+      <x:c r="F81" s="18" t="n">
+        <x:f>D81-E81</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="16"/>
       <x:c r="B82" s="17"/>
       <x:c r="C82" s="23"/>
       <x:c r="D82" s="18"/>
-      <x:c r="E82" s="17"/>
-      <x:c r="F82" s="23"/>
+      <x:c r="E82" s="18"/>
+      <x:c r="F82" s="18" t="n">
+        <x:f>D82-E82</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="16"/>
       <x:c r="B83" s="17"/>
       <x:c r="C83" s="23"/>
       <x:c r="D83" s="18"/>
-      <x:c r="E83" s="17"/>
-      <x:c r="F83" s="23"/>
+      <x:c r="E83" s="18"/>
+      <x:c r="F83" s="18" t="n">
+        <x:f>D83-E83</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="16"/>
       <x:c r="B84" s="17"/>
       <x:c r="C84" s="23"/>
       <x:c r="D84" s="18"/>
-      <x:c r="E84" s="17"/>
-      <x:c r="F84" s="23"/>
+      <x:c r="E84" s="18"/>
+      <x:c r="F84" s="18" t="n">
+        <x:f>D84-E84</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="16"/>
       <x:c r="B85" s="17"/>
       <x:c r="C85" s="23"/>
       <x:c r="D85" s="18"/>
-      <x:c r="E85" s="17"/>
-      <x:c r="F85" s="23"/>
+      <x:c r="E85" s="18"/>
+      <x:c r="F85" s="18" t="n">
+        <x:f>D85-E85</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="16"/>
       <x:c r="B86" s="17"/>
       <x:c r="C86" s="23"/>
       <x:c r="D86" s="18"/>
-      <x:c r="E86" s="17"/>
-      <x:c r="F86" s="23"/>
+      <x:c r="E86" s="18"/>
+      <x:c r="F86" s="18" t="n">
+        <x:f>D86-E86</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="16"/>
       <x:c r="B87" s="17"/>
       <x:c r="C87" s="23"/>
       <x:c r="D87" s="18"/>
-      <x:c r="E87" s="17"/>
-      <x:c r="F87" s="23"/>
+      <x:c r="E87" s="18"/>
+      <x:c r="F87" s="18" t="n">
+        <x:f>D87-E87</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="16"/>
       <x:c r="B88" s="17"/>
       <x:c r="C88" s="23"/>
       <x:c r="D88" s="18"/>
-      <x:c r="E88" s="17"/>
-      <x:c r="F88" s="23"/>
+      <x:c r="E88" s="18"/>
+      <x:c r="F88" s="18" t="n">
+        <x:f>D88-E88</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="16"/>
       <x:c r="B89" s="17"/>
       <x:c r="C89" s="23"/>
       <x:c r="D89" s="18"/>
-      <x:c r="E89" s="17"/>
-      <x:c r="F89" s="23"/>
+      <x:c r="E89" s="18"/>
+      <x:c r="F89" s="18" t="n">
+        <x:f>D89-E89</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="16"/>
       <x:c r="B90" s="17"/>
       <x:c r="C90" s="23"/>
       <x:c r="D90" s="18"/>
-      <x:c r="E90" s="17"/>
-      <x:c r="F90" s="23"/>
+      <x:c r="E90" s="18"/>
+      <x:c r="F90" s="18" t="n">
+        <x:f>D90-E90</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="16"/>
       <x:c r="B91" s="17"/>
       <x:c r="C91" s="23"/>
       <x:c r="D91" s="18"/>
-      <x:c r="E91" s="17"/>
-      <x:c r="F91" s="23"/>
+      <x:c r="E91" s="18"/>
+      <x:c r="F91" s="18" t="n">
+        <x:f>D91-E91</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="16"/>
       <x:c r="B92" s="17"/>
       <x:c r="C92" s="23"/>
       <x:c r="D92" s="18"/>
-      <x:c r="E92" s="17"/>
-      <x:c r="F92" s="23"/>
+      <x:c r="E92" s="18"/>
+      <x:c r="F92" s="18" t="n">
+        <x:f>D92-E92</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="16"/>
       <x:c r="B93" s="17"/>
       <x:c r="C93" s="23"/>
       <x:c r="D93" s="18"/>
-      <x:c r="E93" s="17"/>
-      <x:c r="F93" s="23"/>
+      <x:c r="E93" s="18"/>
+      <x:c r="F93" s="18" t="n">
+        <x:f>D93-E93</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="16"/>
       <x:c r="B94" s="17"/>
       <x:c r="C94" s="23"/>
       <x:c r="D94" s="18"/>
-      <x:c r="E94" s="17"/>
-      <x:c r="F94" s="23"/>
+      <x:c r="E94" s="18"/>
+      <x:c r="F94" s="18" t="n">
+        <x:f>D94-E94</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="16"/>
       <x:c r="B95" s="17"/>
       <x:c r="C95" s="23"/>
       <x:c r="D95" s="18"/>
-      <x:c r="E95" s="17"/>
-      <x:c r="F95" s="23"/>
+      <x:c r="E95" s="18"/>
+      <x:c r="F95" s="18" t="n">
+        <x:f>D95-E95</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="16"/>
       <x:c r="B96" s="17"/>
       <x:c r="C96" s="23"/>
       <x:c r="D96" s="18"/>
-      <x:c r="E96" s="17"/>
-      <x:c r="F96" s="23"/>
+      <x:c r="E96" s="18"/>
+      <x:c r="F96" s="18" t="n">
+        <x:f>D96-E96</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="16"/>
       <x:c r="B97" s="17"/>
       <x:c r="C97" s="23"/>
       <x:c r="D97" s="18"/>
-      <x:c r="E97" s="17"/>
-      <x:c r="F97" s="23"/>
+      <x:c r="E97" s="18"/>
+      <x:c r="F97" s="18" t="n">
+        <x:f>D97-E97</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="16"/>
       <x:c r="B98" s="17"/>
       <x:c r="C98" s="23"/>
       <x:c r="D98" s="18"/>
-      <x:c r="E98" s="17"/>
-      <x:c r="F98" s="23"/>
+      <x:c r="E98" s="18"/>
+      <x:c r="F98" s="18" t="n">
+        <x:f>D98-E98</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="16"/>
       <x:c r="B99" s="17"/>
       <x:c r="C99" s="23"/>
       <x:c r="D99" s="18"/>
-      <x:c r="E99" s="17"/>
-      <x:c r="F99" s="23"/>
+      <x:c r="E99" s="18"/>
+      <x:c r="F99" s="18" t="n">
+        <x:f>D99-E99</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="16"/>
       <x:c r="B100" s="17"/>
       <x:c r="C100" s="23"/>
       <x:c r="D100" s="18"/>
-      <x:c r="E100" s="17"/>
-      <x:c r="F100" s="23"/>
+      <x:c r="E100" s="18"/>
+      <x:c r="F100" s="18" t="n">
+        <x:f>D100-E100</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="16"/>
       <x:c r="B101" s="17"/>
       <x:c r="C101" s="23"/>
       <x:c r="D101" s="18"/>
-      <x:c r="E101" s="17"/>
-      <x:c r="F101" s="23"/>
+      <x:c r="E101" s="18"/>
+      <x:c r="F101" s="18" t="n">
+        <x:f>D101-E101</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="16"/>
       <x:c r="B102" s="17"/>
       <x:c r="C102" s="23"/>
       <x:c r="D102" s="18"/>
-      <x:c r="E102" s="17"/>
-      <x:c r="F102" s="23"/>
+      <x:c r="E102" s="18"/>
+      <x:c r="F102" s="18" t="n">
+        <x:f>D102-E102</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="16"/>
       <x:c r="B103" s="17"/>
       <x:c r="C103" s="23"/>
       <x:c r="D103" s="18"/>
-      <x:c r="E103" s="17"/>
-      <x:c r="F103" s="23"/>
+      <x:c r="E103" s="18"/>
+      <x:c r="F103" s="18" t="n">
+        <x:f>D103-E103</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="16"/>
       <x:c r="B104" s="17"/>
       <x:c r="C104" s="23"/>
       <x:c r="D104" s="18"/>
-      <x:c r="E104" s="17"/>
-      <x:c r="F104" s="23"/>
+      <x:c r="E104" s="18"/>
+      <x:c r="F104" s="18" t="n">
+        <x:f>D104-E104</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="16"/>
       <x:c r="B105" s="17"/>
       <x:c r="C105" s="23"/>
       <x:c r="D105" s="18"/>
-      <x:c r="E105" s="17"/>
-      <x:c r="F105" s="23"/>
+      <x:c r="E105" s="18"/>
+      <x:c r="F105" s="18" t="n">
+        <x:f>D105-E105</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="16"/>
       <x:c r="B106" s="17"/>
       <x:c r="C106" s="23"/>
       <x:c r="D106" s="18"/>
-      <x:c r="E106" s="17"/>
-      <x:c r="F106" s="23"/>
+      <x:c r="E106" s="18"/>
+      <x:c r="F106" s="18" t="n">
+        <x:f>D106-E106</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="16"/>
       <x:c r="B107" s="17"/>
       <x:c r="C107" s="23"/>
       <x:c r="D107" s="18"/>
-      <x:c r="E107" s="17"/>
-      <x:c r="F107" s="23"/>
+      <x:c r="E107" s="18"/>
+      <x:c r="F107" s="18" t="n">
+        <x:f>D107-E107</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="16"/>
       <x:c r="B108" s="17"/>
       <x:c r="C108" s="23"/>
       <x:c r="D108" s="18"/>
-      <x:c r="E108" s="17"/>
-      <x:c r="F108" s="23"/>
+      <x:c r="E108" s="18"/>
+      <x:c r="F108" s="18" t="n">
+        <x:f>D108-E108</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="16"/>
       <x:c r="B109" s="17"/>
       <x:c r="C109" s="23"/>
       <x:c r="D109" s="18"/>
-      <x:c r="E109" s="17"/>
-      <x:c r="F109" s="23"/>
+      <x:c r="E109" s="18"/>
+      <x:c r="F109" s="18" t="n">
+        <x:f>D109-E109</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="16"/>
       <x:c r="B110" s="17"/>
       <x:c r="C110" s="23"/>
       <x:c r="D110" s="18"/>
-      <x:c r="E110" s="17"/>
-      <x:c r="F110" s="23"/>
+      <x:c r="E110" s="18"/>
+      <x:c r="F110" s="18" t="n">
+        <x:f>D110-E110</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="16"/>
       <x:c r="B111" s="17"/>
       <x:c r="C111" s="23"/>
       <x:c r="D111" s="18"/>
-      <x:c r="E111" s="17"/>
-      <x:c r="F111" s="23"/>
+      <x:c r="E111" s="18"/>
+      <x:c r="F111" s="18" t="n">
+        <x:f>D111-E111</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="16"/>
       <x:c r="B112" s="17"/>
       <x:c r="C112" s="23"/>
       <x:c r="D112" s="18"/>
-      <x:c r="E112" s="17"/>
-      <x:c r="F112" s="23"/>
+      <x:c r="E112" s="18"/>
+      <x:c r="F112" s="18" t="n">
+        <x:f>D112-E112</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="16"/>
       <x:c r="B113" s="17"/>
       <x:c r="C113" s="23"/>
       <x:c r="D113" s="18"/>
-      <x:c r="E113" s="17"/>
-      <x:c r="F113" s="23"/>
+      <x:c r="E113" s="18"/>
+      <x:c r="F113" s="18" t="n">
+        <x:f>D113-E113</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="16"/>
       <x:c r="B114" s="17"/>
       <x:c r="C114" s="23"/>
       <x:c r="D114" s="18"/>
-      <x:c r="E114" s="17"/>
-      <x:c r="F114" s="23"/>
+      <x:c r="E114" s="18"/>
+      <x:c r="F114" s="18" t="n">
+        <x:f>D114-E114</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="16"/>
       <x:c r="B115" s="17"/>
       <x:c r="C115" s="23"/>
       <x:c r="D115" s="18"/>
-      <x:c r="E115" s="17"/>
-      <x:c r="F115" s="23"/>
+      <x:c r="E115" s="18"/>
+      <x:c r="F115" s="18" t="n">
+        <x:f>D115-E115</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="16"/>
       <x:c r="B116" s="17"/>
       <x:c r="C116" s="23"/>
       <x:c r="D116" s="18"/>
-      <x:c r="E116" s="17"/>
-      <x:c r="F116" s="23"/>
+      <x:c r="E116" s="18"/>
+      <x:c r="F116" s="18" t="n">
+        <x:f>D116-E116</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="16"/>
       <x:c r="B117" s="17"/>
       <x:c r="C117" s="23"/>
       <x:c r="D117" s="18"/>
-      <x:c r="E117" s="17"/>
-      <x:c r="F117" s="23"/>
+      <x:c r="E117" s="18"/>
+      <x:c r="F117" s="18" t="n">
+        <x:f>D117-E117</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="16"/>
       <x:c r="B118" s="17"/>
       <x:c r="C118" s="23"/>
       <x:c r="D118" s="18"/>
-      <x:c r="E118" s="17"/>
-      <x:c r="F118" s="23"/>
+      <x:c r="E118" s="18"/>
+      <x:c r="F118" s="18" t="n">
+        <x:f>D118-E118</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="16"/>
       <x:c r="B119" s="17"/>
       <x:c r="C119" s="23"/>
       <x:c r="D119" s="18"/>
-      <x:c r="E119" s="17"/>
-      <x:c r="F119" s="23"/>
+      <x:c r="E119" s="18"/>
+      <x:c r="F119" s="18" t="n">
+        <x:f>D119-E119</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="16"/>
       <x:c r="B120" s="17"/>
       <x:c r="C120" s="23"/>
       <x:c r="D120" s="18"/>
-      <x:c r="E120" s="17"/>
-      <x:c r="F120" s="23"/>
+      <x:c r="E120" s="18"/>
+      <x:c r="F120" s="18" t="n">
+        <x:f>D120-E120</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="16"/>
       <x:c r="B121" s="17"/>
       <x:c r="C121" s="23"/>
       <x:c r="D121" s="18"/>
-      <x:c r="E121" s="17"/>
-      <x:c r="F121" s="23"/>
+      <x:c r="E121" s="18"/>
+      <x:c r="F121" s="18" t="n">
+        <x:f>D121-E121</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="16"/>
       <x:c r="B122" s="17"/>
       <x:c r="C122" s="23"/>
       <x:c r="D122" s="18"/>
-      <x:c r="E122" s="17"/>
-      <x:c r="F122" s="23"/>
+      <x:c r="E122" s="18"/>
+      <x:c r="F122" s="18" t="n">
+        <x:f>D122-E122</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="16"/>
       <x:c r="B123" s="17"/>
       <x:c r="C123" s="23"/>
       <x:c r="D123" s="18"/>
-      <x:c r="E123" s="17"/>
-      <x:c r="F123" s="23"/>
+      <x:c r="E123" s="18"/>
+      <x:c r="F123" s="18" t="n">
+        <x:f>D123-E123</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="16"/>
       <x:c r="B124" s="17"/>
       <x:c r="C124" s="23"/>
       <x:c r="D124" s="18"/>
-      <x:c r="E124" s="17"/>
-      <x:c r="F124" s="23"/>
+      <x:c r="E124" s="18"/>
+      <x:c r="F124" s="18" t="n">
+        <x:f>D124-E124</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="16"/>
       <x:c r="B125" s="17"/>
       <x:c r="C125" s="23"/>
       <x:c r="D125" s="18"/>
-      <x:c r="E125" s="17"/>
-      <x:c r="F125" s="23"/>
+      <x:c r="E125" s="18"/>
+      <x:c r="F125" s="18" t="n">
+        <x:f>D125-E125</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="16"/>
       <x:c r="B126" s="17"/>
       <x:c r="C126" s="23"/>
       <x:c r="D126" s="18"/>
-      <x:c r="E126" s="17"/>
-      <x:c r="F126" s="23"/>
+      <x:c r="E126" s="18"/>
+      <x:c r="F126" s="18" t="n">
+        <x:f>D126-E126</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="16"/>
       <x:c r="B127" s="17"/>
       <x:c r="C127" s="23"/>
       <x:c r="D127" s="18"/>
-      <x:c r="E127" s="17"/>
-      <x:c r="F127" s="23"/>
+      <x:c r="E127" s="18"/>
+      <x:c r="F127" s="18" t="n">
+        <x:f>D127-E127</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="16"/>
       <x:c r="B128" s="17"/>
       <x:c r="C128" s="23"/>
       <x:c r="D128" s="18"/>
-      <x:c r="E128" s="17"/>
-      <x:c r="F128" s="23"/>
+      <x:c r="E128" s="18"/>
+      <x:c r="F128" s="18" t="n">
+        <x:f>D128-E128</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="16"/>
       <x:c r="B129" s="17"/>
       <x:c r="C129" s="23"/>
       <x:c r="D129" s="18"/>
-      <x:c r="E129" s="17"/>
-      <x:c r="F129" s="23"/>
+      <x:c r="E129" s="18"/>
+      <x:c r="F129" s="18" t="n">
+        <x:f>D129-E129</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="16"/>
       <x:c r="B130" s="17"/>
       <x:c r="C130" s="23"/>
       <x:c r="D130" s="18"/>
-      <x:c r="E130" s="17"/>
-      <x:c r="F130" s="23"/>
+      <x:c r="E130" s="18"/>
+      <x:c r="F130" s="18" t="n">
+        <x:f>D130-E130</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="16"/>
       <x:c r="B131" s="17"/>
       <x:c r="C131" s="23"/>
       <x:c r="D131" s="18"/>
-      <x:c r="E131" s="17"/>
-      <x:c r="F131" s="23"/>
+      <x:c r="E131" s="18"/>
+      <x:c r="F131" s="18" t="n">
+        <x:f>D131-E131</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="16"/>
       <x:c r="B132" s="17"/>
       <x:c r="C132" s="23"/>
       <x:c r="D132" s="18"/>
-      <x:c r="E132" s="17"/>
-      <x:c r="F132" s="23"/>
+      <x:c r="E132" s="18"/>
+      <x:c r="F132" s="18" t="n">
+        <x:f>D132-E132</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="16"/>
       <x:c r="B133" s="17"/>
       <x:c r="C133" s="23"/>
       <x:c r="D133" s="18"/>
-      <x:c r="E133" s="17"/>
-      <x:c r="F133" s="23"/>
+      <x:c r="E133" s="18"/>
+      <x:c r="F133" s="18" t="n">
+        <x:f>D133-E133</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="16"/>
       <x:c r="B134" s="17"/>
       <x:c r="C134" s="23"/>
       <x:c r="D134" s="18"/>
-      <x:c r="E134" s="17"/>
-      <x:c r="F134" s="23"/>
+      <x:c r="E134" s="18"/>
+      <x:c r="F134" s="18" t="n">
+        <x:f>D134-E134</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="16"/>
       <x:c r="B135" s="17"/>
       <x:c r="C135" s="23"/>
       <x:c r="D135" s="18"/>
-      <x:c r="E135" s="17"/>
-      <x:c r="F135" s="23"/>
+      <x:c r="E135" s="18"/>
+      <x:c r="F135" s="18" t="n">
+        <x:f>D135-E135</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="16"/>
       <x:c r="B136" s="17"/>
       <x:c r="C136" s="23"/>
       <x:c r="D136" s="18"/>
-      <x:c r="E136" s="17"/>
-      <x:c r="F136" s="23"/>
+      <x:c r="E136" s="18"/>
+      <x:c r="F136" s="18" t="n">
+        <x:f>D136-E136</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="16"/>
       <x:c r="B137" s="17"/>
       <x:c r="C137" s="23"/>
       <x:c r="D137" s="18"/>
-      <x:c r="E137" s="17"/>
-      <x:c r="F137" s="23"/>
+      <x:c r="E137" s="18"/>
+      <x:c r="F137" s="18" t="n">
+        <x:f>D137-E137</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="16"/>
       <x:c r="B138" s="17"/>
       <x:c r="C138" s="23"/>
       <x:c r="D138" s="18"/>
-      <x:c r="E138" s="17"/>
-      <x:c r="F138" s="23"/>
+      <x:c r="E138" s="18"/>
+      <x:c r="F138" s="18" t="n">
+        <x:f>D138-E138</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="16"/>
       <x:c r="B139" s="17"/>
       <x:c r="C139" s="23"/>
       <x:c r="D139" s="18"/>
-      <x:c r="E139" s="17"/>
-      <x:c r="F139" s="23"/>
+      <x:c r="E139" s="18"/>
+      <x:c r="F139" s="18" t="n">
+        <x:f>D139-E139</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="16"/>
       <x:c r="B140" s="17"/>
       <x:c r="C140" s="23"/>
       <x:c r="D140" s="18"/>
-      <x:c r="E140" s="17"/>
-      <x:c r="F140" s="23"/>
+      <x:c r="E140" s="18"/>
+      <x:c r="F140" s="18" t="n">
+        <x:f>D140-E140</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="16"/>
       <x:c r="B141" s="17"/>
       <x:c r="C141" s="23"/>
       <x:c r="D141" s="18"/>
-      <x:c r="E141" s="17"/>
-      <x:c r="F141" s="23"/>
+      <x:c r="E141" s="18"/>
+      <x:c r="F141" s="18" t="n">
+        <x:f>D141-E141</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="16"/>
       <x:c r="B142" s="17"/>
       <x:c r="C142" s="23"/>
       <x:c r="D142" s="18"/>
-      <x:c r="E142" s="17"/>
-      <x:c r="F142" s="23"/>
+      <x:c r="E142" s="18"/>
+      <x:c r="F142" s="18" t="n">
+        <x:f>D142-E142</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="16"/>
       <x:c r="B143" s="17"/>
       <x:c r="C143" s="23"/>
       <x:c r="D143" s="18"/>
-      <x:c r="E143" s="17"/>
-      <x:c r="F143" s="23"/>
+      <x:c r="E143" s="18"/>
+      <x:c r="F143" s="18" t="n">
+        <x:f>D143-E143</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="16"/>
       <x:c r="B144" s="17"/>
       <x:c r="C144" s="23"/>
       <x:c r="D144" s="18"/>
-      <x:c r="E144" s="17"/>
-      <x:c r="F144" s="23"/>
+      <x:c r="E144" s="18"/>
+      <x:c r="F144" s="18" t="n">
+        <x:f>D144-E144</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="16"/>
       <x:c r="B145" s="17"/>
       <x:c r="C145" s="23"/>
       <x:c r="D145" s="18"/>
-      <x:c r="E145" s="17"/>
-      <x:c r="F145" s="23"/>
+      <x:c r="E145" s="18"/>
+      <x:c r="F145" s="18" t="n">
+        <x:f>D145-E145</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="16"/>
       <x:c r="B146" s="17"/>
       <x:c r="C146" s="23"/>
       <x:c r="D146" s="18"/>
-      <x:c r="E146" s="17"/>
-      <x:c r="F146" s="23"/>
+      <x:c r="E146" s="18"/>
+      <x:c r="F146" s="18" t="n">
+        <x:f>D146-E146</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="16"/>
       <x:c r="B147" s="17"/>
       <x:c r="C147" s="23"/>
       <x:c r="D147" s="18"/>
-      <x:c r="E147" s="17"/>
-      <x:c r="F147" s="23"/>
+      <x:c r="E147" s="18"/>
+      <x:c r="F147" s="18" t="n">
+        <x:f>D147-E147</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="16"/>
       <x:c r="B148" s="17"/>
       <x:c r="C148" s="23"/>
       <x:c r="D148" s="18"/>
-      <x:c r="E148" s="17"/>
-      <x:c r="F148" s="23"/>
+      <x:c r="E148" s="18"/>
+      <x:c r="F148" s="18" t="n">
+        <x:f>D148-E148</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="16"/>
       <x:c r="B149" s="17"/>
       <x:c r="C149" s="23"/>
       <x:c r="D149" s="18"/>
-      <x:c r="E149" s="17"/>
-      <x:c r="F149" s="23"/>
+      <x:c r="E149" s="18"/>
+      <x:c r="F149" s="18" t="n">
+        <x:f>D149-E149</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="16"/>
       <x:c r="B150" s="17"/>
       <x:c r="C150" s="23"/>
       <x:c r="D150" s="18"/>
-      <x:c r="E150" s="17"/>
-      <x:c r="F150" s="23"/>
+      <x:c r="E150" s="18"/>
+      <x:c r="F150" s="18" t="n">
+        <x:f>D150-E150</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="16"/>
       <x:c r="B151" s="17"/>
       <x:c r="C151" s="23"/>
       <x:c r="D151" s="18"/>
-      <x:c r="E151" s="17"/>
-      <x:c r="F151" s="23"/>
+      <x:c r="E151" s="18"/>
+      <x:c r="F151" s="18" t="n">
+        <x:f>D151-E151</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="16"/>
       <x:c r="B152" s="17"/>
       <x:c r="C152" s="23"/>
       <x:c r="D152" s="18"/>
-      <x:c r="E152" s="17"/>
-      <x:c r="F152" s="23"/>
+      <x:c r="E152" s="18"/>
+      <x:c r="F152" s="18" t="n">
+        <x:f>D152-E152</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="16"/>
       <x:c r="B153" s="17"/>
       <x:c r="C153" s="23"/>
       <x:c r="D153" s="18"/>
-      <x:c r="E153" s="17"/>
-      <x:c r="F153" s="23"/>
+      <x:c r="E153" s="18"/>
+      <x:c r="F153" s="18" t="n">
+        <x:f>D153-E153</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="16"/>
       <x:c r="B154" s="17"/>
       <x:c r="C154" s="23"/>
       <x:c r="D154" s="18"/>
-      <x:c r="E154" s="17"/>
-      <x:c r="F154" s="23"/>
+      <x:c r="E154" s="18"/>
+      <x:c r="F154" s="18" t="n">
+        <x:f>D154-E154</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="16"/>
       <x:c r="B155" s="17"/>
       <x:c r="C155" s="23"/>
       <x:c r="D155" s="18"/>
-      <x:c r="E155" s="17"/>
-      <x:c r="F155" s="23"/>
+      <x:c r="E155" s="18"/>
+      <x:c r="F155" s="18" t="n">
+        <x:f>D155-E155</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="16"/>
       <x:c r="B156" s="17"/>
       <x:c r="C156" s="23"/>
       <x:c r="D156" s="18"/>
-      <x:c r="E156" s="17"/>
-      <x:c r="F156" s="23"/>
+      <x:c r="E156" s="18"/>
+      <x:c r="F156" s="18" t="n">
+        <x:f>D156-E156</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="16"/>
       <x:c r="B157" s="17"/>
       <x:c r="C157" s="23"/>
       <x:c r="D157" s="18"/>
-      <x:c r="E157" s="17"/>
-      <x:c r="F157" s="23"/>
+      <x:c r="E157" s="18"/>
+      <x:c r="F157" s="18" t="n">
+        <x:f>D157-E157</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="16"/>
       <x:c r="B158" s="17"/>
       <x:c r="C158" s="23"/>
       <x:c r="D158" s="18"/>
-      <x:c r="E158" s="17"/>
-      <x:c r="F158" s="23"/>
+      <x:c r="E158" s="18"/>
+      <x:c r="F158" s="18" t="n">
+        <x:f>D158-E158</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="16"/>
       <x:c r="B159" s="17"/>
       <x:c r="C159" s="23"/>
       <x:c r="D159" s="18"/>
-      <x:c r="E159" s="17"/>
-      <x:c r="F159" s="23"/>
+      <x:c r="E159" s="18"/>
+      <x:c r="F159" s="18" t="n">
+        <x:f>D159-E159</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="16"/>
       <x:c r="B160" s="17"/>
       <x:c r="C160" s="23"/>
       <x:c r="D160" s="18"/>
-      <x:c r="E160" s="17"/>
-      <x:c r="F160" s="23"/>
+      <x:c r="E160" s="18"/>
+      <x:c r="F160" s="18" t="n">
+        <x:f>D160-E160</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="16"/>
       <x:c r="B161" s="17"/>
       <x:c r="C161" s="23"/>
       <x:c r="D161" s="18"/>
-      <x:c r="E161" s="17"/>
-      <x:c r="F161" s="23"/>
+      <x:c r="E161" s="18"/>
+      <x:c r="F161" s="18" t="n">
+        <x:f>D161-E161</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="16"/>
       <x:c r="B162" s="17"/>
       <x:c r="C162" s="23"/>
       <x:c r="D162" s="18"/>
-      <x:c r="E162" s="17"/>
-      <x:c r="F162" s="23"/>
+      <x:c r="E162" s="18"/>
+      <x:c r="F162" s="18" t="n">
+        <x:f>D162-E162</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="16"/>
       <x:c r="B163" s="17"/>
       <x:c r="C163" s="23"/>
       <x:c r="D163" s="18"/>
-      <x:c r="E163" s="17"/>
-      <x:c r="F163" s="23"/>
+      <x:c r="E163" s="18"/>
+      <x:c r="F163" s="18" t="n">
+        <x:f>D163-E163</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="16"/>
       <x:c r="B164" s="17"/>
       <x:c r="C164" s="23"/>
       <x:c r="D164" s="18"/>
-      <x:c r="E164" s="17"/>
-      <x:c r="F164" s="23"/>
+      <x:c r="E164" s="18"/>
+      <x:c r="F164" s="18" t="n">
+        <x:f>D164-E164</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="16"/>
       <x:c r="B165" s="17"/>
       <x:c r="C165" s="23"/>
       <x:c r="D165" s="18"/>
-      <x:c r="E165" s="17"/>
-      <x:c r="F165" s="23"/>
+      <x:c r="E165" s="18"/>
+      <x:c r="F165" s="18" t="n">
+        <x:f>D165-E165</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="16"/>
       <x:c r="B166" s="17"/>
       <x:c r="C166" s="23"/>
       <x:c r="D166" s="18"/>
-      <x:c r="E166" s="17"/>
-      <x:c r="F166" s="23"/>
+      <x:c r="E166" s="18"/>
+      <x:c r="F166" s="18" t="n">
+        <x:f>D166-E166</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="16"/>
       <x:c r="B167" s="17"/>
       <x:c r="C167" s="23"/>
       <x:c r="D167" s="18"/>
-      <x:c r="E167" s="17"/>
-      <x:c r="F167" s="23"/>
+      <x:c r="E167" s="18"/>
+      <x:c r="F167" s="18" t="n">
+        <x:f>D167-E167</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="16"/>
       <x:c r="B168" s="17"/>
       <x:c r="C168" s="23"/>
       <x:c r="D168" s="18"/>
-      <x:c r="E168" s="17"/>
-      <x:c r="F168" s="23"/>
+      <x:c r="E168" s="18"/>
+      <x:c r="F168" s="18" t="n">
+        <x:f>D168-E168</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="16"/>
       <x:c r="B169" s="17"/>
       <x:c r="C169" s="23"/>
       <x:c r="D169" s="18"/>
-      <x:c r="E169" s="17"/>
-      <x:c r="F169" s="23"/>
+      <x:c r="E169" s="18"/>
+      <x:c r="F169" s="18" t="n">
+        <x:f>D169-E169</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="16"/>
       <x:c r="B170" s="17"/>
       <x:c r="C170" s="23"/>
       <x:c r="D170" s="18"/>
-      <x:c r="E170" s="17"/>
-      <x:c r="F170" s="23"/>
+      <x:c r="E170" s="18"/>
+      <x:c r="F170" s="18" t="n">
+        <x:f>D170-E170</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="16"/>
       <x:c r="B171" s="17"/>
       <x:c r="C171" s="23"/>
       <x:c r="D171" s="18"/>
-      <x:c r="E171" s="17"/>
-      <x:c r="F171" s="23"/>
+      <x:c r="E171" s="18"/>
+      <x:c r="F171" s="18" t="n">
+        <x:f>D171-E171</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="16"/>
       <x:c r="B172" s="17"/>
       <x:c r="C172" s="23"/>
       <x:c r="D172" s="18"/>
-      <x:c r="E172" s="17"/>
-      <x:c r="F172" s="23"/>
+      <x:c r="E172" s="18"/>
+      <x:c r="F172" s="18" t="n">
+        <x:f>D172-E172</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="16"/>
       <x:c r="B173" s="17"/>
       <x:c r="C173" s="23"/>
       <x:c r="D173" s="18"/>
-      <x:c r="E173" s="17"/>
-      <x:c r="F173" s="23"/>
+      <x:c r="E173" s="18"/>
+      <x:c r="F173" s="18" t="n">
+        <x:f>D173-E173</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="16"/>
       <x:c r="B174" s="17"/>
       <x:c r="C174" s="23"/>
       <x:c r="D174" s="18"/>
-      <x:c r="E174" s="17"/>
-      <x:c r="F174" s="23"/>
+      <x:c r="E174" s="18"/>
+      <x:c r="F174" s="18" t="n">
+        <x:f>D174-E174</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="16"/>
       <x:c r="B175" s="17"/>
       <x:c r="C175" s="23"/>
       <x:c r="D175" s="18"/>
-      <x:c r="E175" s="17"/>
-      <x:c r="F175" s="23"/>
+      <x:c r="E175" s="18"/>
+      <x:c r="F175" s="18" t="n">
+        <x:f>D175-E175</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="16"/>
       <x:c r="B176" s="17"/>
       <x:c r="C176" s="23"/>
       <x:c r="D176" s="18"/>
-      <x:c r="E176" s="17"/>
-      <x:c r="F176" s="23"/>
+      <x:c r="E176" s="18"/>
+      <x:c r="F176" s="18" t="n">
+        <x:f>D176-E176</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="16"/>
       <x:c r="B177" s="17"/>
       <x:c r="C177" s="23"/>
       <x:c r="D177" s="18"/>
-      <x:c r="E177" s="17"/>
-      <x:c r="F177" s="23"/>
+      <x:c r="E177" s="18"/>
+      <x:c r="F177" s="18" t="n">
+        <x:f>D177-E177</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="16"/>
       <x:c r="B178" s="17"/>
       <x:c r="C178" s="23"/>
       <x:c r="D178" s="18"/>
-      <x:c r="E178" s="17"/>
-      <x:c r="F178" s="23"/>
+      <x:c r="E178" s="18"/>
+      <x:c r="F178" s="18" t="n">
+        <x:f>D178-E178</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="16"/>
       <x:c r="B179" s="17"/>
       <x:c r="C179" s="23"/>
       <x:c r="D179" s="18"/>
-      <x:c r="E179" s="17"/>
-      <x:c r="F179" s="23"/>
+      <x:c r="E179" s="18"/>
+      <x:c r="F179" s="18" t="n">
+        <x:f>D179-E179</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="16"/>
       <x:c r="B180" s="17"/>
       <x:c r="C180" s="23"/>
       <x:c r="D180" s="18"/>
-      <x:c r="E180" s="17"/>
-      <x:c r="F180" s="23"/>
+      <x:c r="E180" s="18"/>
+      <x:c r="F180" s="18" t="n">
+        <x:f>D180-E180</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="16"/>
       <x:c r="B181" s="17"/>
       <x:c r="C181" s="23"/>
       <x:c r="D181" s="18"/>
-      <x:c r="E181" s="17"/>
-      <x:c r="F181" s="23"/>
+      <x:c r="E181" s="18"/>
+      <x:c r="F181" s="18" t="n">
+        <x:f>D181-E181</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="16"/>
       <x:c r="B182" s="17"/>
       <x:c r="C182" s="23"/>
       <x:c r="D182" s="18"/>
-      <x:c r="E182" s="17"/>
-      <x:c r="F182" s="23"/>
+      <x:c r="E182" s="18"/>
+      <x:c r="F182" s="18" t="n">
+        <x:f>D182-E182</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="16"/>
       <x:c r="B183" s="17"/>
       <x:c r="C183" s="23"/>
       <x:c r="D183" s="18"/>
-      <x:c r="E183" s="17"/>
-      <x:c r="F183" s="23"/>
+      <x:c r="E183" s="18"/>
+      <x:c r="F183" s="18" t="n">
+        <x:f>D183-E183</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="16"/>
       <x:c r="B184" s="17"/>
       <x:c r="C184" s="23"/>
       <x:c r="D184" s="18"/>
-      <x:c r="E184" s="17"/>
-      <x:c r="F184" s="23"/>
+      <x:c r="E184" s="18"/>
+      <x:c r="F184" s="18" t="n">
+        <x:f>D184-E184</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="16"/>
       <x:c r="B185" s="17"/>
       <x:c r="C185" s="23"/>
       <x:c r="D185" s="18"/>
-      <x:c r="E185" s="17"/>
-      <x:c r="F185" s="23"/>
+      <x:c r="E185" s="18"/>
+      <x:c r="F185" s="18" t="n">
+        <x:f>D185-E185</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="16"/>
       <x:c r="B186" s="17"/>
       <x:c r="C186" s="23"/>
       <x:c r="D186" s="18"/>
-      <x:c r="E186" s="17"/>
-      <x:c r="F186" s="23"/>
+      <x:c r="E186" s="18"/>
+      <x:c r="F186" s="18" t="n">
+        <x:f>D186-E186</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="16"/>
       <x:c r="B187" s="17"/>
       <x:c r="C187" s="23"/>
       <x:c r="D187" s="18"/>
-      <x:c r="E187" s="17"/>
-      <x:c r="F187" s="23"/>
+      <x:c r="E187" s="18"/>
+      <x:c r="F187" s="18" t="n">
+        <x:f>D187-E187</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="16"/>
       <x:c r="B188" s="17"/>
       <x:c r="C188" s="23"/>
       <x:c r="D188" s="18"/>
-      <x:c r="E188" s="17"/>
-      <x:c r="F188" s="23"/>
+      <x:c r="E188" s="18"/>
+      <x:c r="F188" s="18" t="n">
+        <x:f>D188-E188</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="16"/>
       <x:c r="B189" s="17"/>
       <x:c r="C189" s="23"/>
       <x:c r="D189" s="18"/>
-      <x:c r="E189" s="17"/>
-      <x:c r="F189" s="23"/>
+      <x:c r="E189" s="18"/>
+      <x:c r="F189" s="18" t="n">
+        <x:f>D189-E189</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="16"/>
       <x:c r="B190" s="17"/>
       <x:c r="C190" s="23"/>
       <x:c r="D190" s="18"/>
-      <x:c r="E190" s="17"/>
-      <x:c r="F190" s="23"/>
+      <x:c r="E190" s="18"/>
+      <x:c r="F190" s="18" t="n">
+        <x:f>D190-E190</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="16"/>
       <x:c r="B191" s="17"/>
       <x:c r="C191" s="23"/>
       <x:c r="D191" s="18"/>
-      <x:c r="E191" s="17"/>
-      <x:c r="F191" s="23"/>
+      <x:c r="E191" s="18"/>
+      <x:c r="F191" s="18" t="n">
+        <x:f>D191-E191</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="16"/>
       <x:c r="B192" s="17"/>
       <x:c r="C192" s="23"/>
       <x:c r="D192" s="18"/>
-      <x:c r="E192" s="17"/>
-      <x:c r="F192" s="23"/>
+      <x:c r="E192" s="18"/>
+      <x:c r="F192" s="18" t="n">
+        <x:f>D192-E192</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="16"/>
       <x:c r="B193" s="17"/>
       <x:c r="C193" s="23"/>
       <x:c r="D193" s="18"/>
-      <x:c r="E193" s="17"/>
-      <x:c r="F193" s="23"/>
+      <x:c r="E193" s="18"/>
+      <x:c r="F193" s="18" t="n">
+        <x:f>D193-E193</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="16"/>
       <x:c r="B194" s="17"/>
       <x:c r="C194" s="23"/>
       <x:c r="D194" s="18"/>
-      <x:c r="E194" s="17"/>
-      <x:c r="F194" s="23"/>
+      <x:c r="E194" s="18"/>
+      <x:c r="F194" s="18" t="n">
+        <x:f>D194-E194</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="16"/>
       <x:c r="B195" s="17"/>
       <x:c r="C195" s="23"/>
       <x:c r="D195" s="18"/>
-      <x:c r="E195" s="17"/>
-      <x:c r="F195" s="23"/>
+      <x:c r="E195" s="18"/>
+      <x:c r="F195" s="18" t="n">
+        <x:f>D195-E195</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="16"/>
       <x:c r="B196" s="17"/>
       <x:c r="C196" s="23"/>
       <x:c r="D196" s="18"/>
-      <x:c r="E196" s="17"/>
-      <x:c r="F196" s="23"/>
+      <x:c r="E196" s="18"/>
+      <x:c r="F196" s="18" t="n">
+        <x:f>D196-E196</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="16"/>
       <x:c r="B197" s="17"/>
       <x:c r="C197" s="23"/>
       <x:c r="D197" s="18"/>
-      <x:c r="E197" s="17"/>
-      <x:c r="F197" s="23"/>
+      <x:c r="E197" s="18"/>
+      <x:c r="F197" s="18" t="n">
+        <x:f>D197-E197</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="16"/>
       <x:c r="B198" s="17"/>
       <x:c r="C198" s="23"/>
       <x:c r="D198" s="18"/>
-      <x:c r="E198" s="17"/>
-      <x:c r="F198" s="23"/>
+      <x:c r="E198" s="18"/>
+      <x:c r="F198" s="18" t="n">
+        <x:f>D198-E198</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="16"/>
       <x:c r="B199" s="17"/>
       <x:c r="C199" s="23"/>
       <x:c r="D199" s="18"/>
-      <x:c r="E199" s="17"/>
-      <x:c r="F199" s="23"/>
+      <x:c r="E199" s="18"/>
+      <x:c r="F199" s="18" t="n">
+        <x:f>D199-E199</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="19"/>
       <x:c r="B200" s="20"/>
       <x:c r="C200" s="24"/>
       <x:c r="D200" s="21"/>
-      <x:c r="E200" s="20"/>
-      <x:c r="F200" s="24"/>
+      <x:c r="E200" s="21"/>
+      <x:c r="F200" s="21" t="n">
+        <x:f>D200-E200</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B2:B200">
-      <x:formula1>"Rent,Staff Salaries,Utilities,Products &amp; Supplies,Equipment,Marketing,Food &amp; Tea,Miscellaneous"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E2:E200">
-      <x:formula1>"Cash,JazzCash,EasyPaisa,Bank Transfer,Card"</x:formula1>
+      <x:formula1>"Rent,Staff Salaries,Utilities,Products &amp; Supplies,Equipment,Marketing,Food &amp; Tea,Miscellaneous,Services,POS Sales,Other Income"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2047,22 +2637,22 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
       <x:c r="B1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
       <x:c r="C1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
       <x:c r="D1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
       <x:c r="E1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
       <x:c r="F1" s="26" t="str">
-        <x:v>Werzio Cash Flow Expense Import Template</x:v>
+        <x:v>Werzio Cash Flow Import Template</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2086,59 +2676,59 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B5" s="31" t="str">
-        <x:v>Required. Select one of the provided category values.</x:v>
+        <x:v>Required. Expense rows must use one of the expense categories provided.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5" t="str">
-        <x:v>Description</x:v>
+        <x:v>Service Description</x:v>
       </x:c>
       <x:c r="B6" s="31" t="str">
-        <x:v>Required. Brief explanation of the expense.</x:v>
+        <x:v>Required. Brief explanation of the service, sale, or expense.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="str">
-        <x:v>Amount (PKR)</x:v>
+        <x:v>Income Intake Amount</x:v>
       </x:c>
       <x:c r="B7" s="31" t="str">
-        <x:v>Required. Positive number without currency symbols.</x:v>
+        <x:v>Enter income here; use 0 for expense-only rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="str">
-        <x:v>Payment Method</x:v>
+        <x:v>Expense Amount</x:v>
       </x:c>
       <x:c r="B8" s="31" t="str">
-        <x:v>Required. Select one of the provided payment values.</x:v>
+        <x:v>Enter expense here; use 0 for income-only rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="str">
-        <x:v>Notes</x:v>
+        <x:v>Closing</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>Optional.</x:v>
+        <x:v>Calculated automatically as Income Intake Amount minus Expense Amount. Do not edit.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="E11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
-        <x:v>Delete the sample rows on the Expenses sheet, add your own records, then upload the workbook from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>